<commit_message>
messages inside the excel are decrypted
</commit_message>
<xml_diff>
--- a/GFGsheet.xlsx
+++ b/GFGsheet.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="44">
   <si>
     <t>0�?v???0 ?	*�H��@@ -155,6 +155,9 @@
   </si>
   <si>
     <t>message from user 3</t>
+  </si>
+  <si>
+    <t>i dont like the TV</t>
   </si>
 </sst>
 </file>
@@ -199,22 +202,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C4"/>
+  <dimension ref="D1:F4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
-      <c r="C1" t="s">
-        <v>42</v>
+      <c r="F1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>42</v>
+      <c r="D2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" t="s">
-        <v>42</v>
+      <c r="E4" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
improve writting to file and reading
</commit_message>
<xml_diff>
--- a/GFGsheet.xlsx
+++ b/GFGsheet.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
   <si>
     <t>0�?v???0 ?	*�H��@@ -202,21 +202,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="D1:F4"/>
+  <dimension ref="G1:L4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
-      <c r="F1" t="s">
+      <c r="I1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L1" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="2">
-      <c r="D2" t="s">
+      <c r="G2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="4">
-      <c r="E4" t="s">
+      <c r="H4" t="s">
+        <v>43</v>
+      </c>
+      <c r="K4" t="s">
         <v>43</v>
       </c>
     </row>

</xml_diff>

<commit_message>
reading messages from file & database
</commit_message>
<xml_diff>
--- a/GFGsheet.xlsx
+++ b/GFGsheet.xlsx
@@ -12,9 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="2">
   <si>
     <t>a message form vimpeli</t>
+  </si>
+  <si>
+    <t>a message form zeriab@hotmail.com</t>
   </si>
 </sst>
 </file>
@@ -59,7 +62,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -72,6 +75,12 @@
       <c r="I1" t="s">
         <v>0</v>
       </c>
+      <c r="L1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O1" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -82,6 +91,12 @@
       </c>
       <c r="G2" t="s">
         <v>0</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1</v>
+      </c>
+      <c r="M2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -94,6 +109,12 @@
       <c r="H4" t="s">
         <v>0</v>
       </c>
+      <c r="K4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N4" t="s">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
implementing an automatic message
</commit_message>
<xml_diff>
--- a/GFGsheet.xlsx
+++ b/GFGsheet.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="2">
   <si>
     <t>a message form vimpeli</t>
   </si>
@@ -62,7 +62,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -79,6 +79,12 @@
         <v>1</v>
       </c>
       <c r="O1" t="s">
+        <v>1</v>
+      </c>
+      <c r="R1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U1" t="s">
         <v>1</v>
       </c>
     </row>
@@ -98,6 +104,12 @@
       <c r="M2" t="s">
         <v>1</v>
       </c>
+      <c r="P2" t="s">
+        <v>1</v>
+      </c>
+      <c r="S2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="s">
@@ -115,6 +127,12 @@
       <c r="N4" t="s">
         <v>1</v>
       </c>
+      <c r="Q4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T4" t="s">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>